<commit_message>
tesztesetek készítése playwright segítségével, dokumentáció megírása hozzá
</commit_message>
<xml_diff>
--- a/projekt/TollUtdij 2025.12/SimiczZalan_TesztDokumentacio.xlsx
+++ b/projekt/TollUtdij 2025.12/SimiczZalan_TesztDokumentacio.xlsx
@@ -5,23 +5,23 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zalan\OneDrive\Asztali gép\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zalan\Dokumentumok\GitHub\13_S2_1_Vizsgaremek2\projekt\TollUtdij 2025.12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A749B1AC-91E2-4323-90A9-AF378B18A7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{449CB01D-B208-4811-9534-B0522AAFB308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{70D12CFA-6C56-45B5-81A0-8FA42F16DDE9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{70D12CFA-6C56-45B5-81A0-8FA42F16DDE9}"/>
   </bookViews>
   <sheets>
-    <sheet name="TesztEset1" sheetId="1" r:id="rId1"/>
-    <sheet name="TesztEset2" sheetId="2" r:id="rId2"/>
-    <sheet name="TesztEset3" sheetId="3" r:id="rId3"/>
-    <sheet name="TesztEset4" sheetId="4" r:id="rId4"/>
-    <sheet name="TesztEset5" sheetId="5" r:id="rId5"/>
-    <sheet name="TesztEset6" sheetId="7" r:id="rId6"/>
-    <sheet name="TesztEset8" sheetId="8" r:id="rId7"/>
-    <sheet name="TesztEset9" sheetId="9" r:id="rId8"/>
-    <sheet name="TesztEset10" sheetId="10" r:id="rId9"/>
+    <sheet name="TesztEset10" sheetId="10" r:id="rId1"/>
+    <sheet name="TesztEset1" sheetId="1" r:id="rId2"/>
+    <sheet name="TesztEset2" sheetId="2" r:id="rId3"/>
+    <sheet name="TesztEset3" sheetId="3" r:id="rId4"/>
+    <sheet name="TesztEset4" sheetId="4" r:id="rId5"/>
+    <sheet name="TesztEset5" sheetId="5" r:id="rId6"/>
+    <sheet name="TesztEset6" sheetId="7" r:id="rId7"/>
+    <sheet name="TesztEset8" sheetId="8" r:id="rId8"/>
+    <sheet name="TesztEset9" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="77">
   <si>
     <t>Mező</t>
   </si>
@@ -74,87 +74,32 @@
     <t>Test Script Test - Tényleges eredmény (Actual Result):</t>
   </si>
   <si>
-    <t>The cart should not contain any items.</t>
-  </si>
-  <si>
     <t>draft</t>
   </si>
   <si>
-    <t>Check the optional operation of cart functions.</t>
-  </si>
-  <si>
     <t>Nagy Huba Kende</t>
   </si>
   <si>
-    <t>30 seconds</t>
-  </si>
-  <si>
-    <t>1.Open https://academybugs.com
-2.Click the Find Bugs link on the navigation bar
-3.Open a product
-4.Open the cart at the bottom of right side menu
-5.Clear the cart if there are any items</t>
-  </si>
-  <si>
     <t>Not necessary</t>
-  </si>
-  <si>
-    <t>The caption of the "Return to Store" button is written with even spacing between letters</t>
-  </si>
-  <si>
-    <t>There is too much space before the last letter in "Return to Store"</t>
-  </si>
-  <si>
-    <t>Number of shown results test</t>
-  </si>
-  <si>
-    <t>Cart test</t>
   </si>
   <si>
     <t>Open https://academybugs.com
 Click the Find Bugs link on the navigation bar</t>
   </si>
   <si>
-    <t>Make sure every function woks on the main page.</t>
-  </si>
-  <si>
     <t>High severity</t>
   </si>
   <si>
     <t>Low severity</t>
   </si>
   <si>
-    <t>Click on the buttons to show a certain number of results at the top left</t>
-  </si>
-  <si>
-    <t>The selected number of results is displayed according to the clicked buttons</t>
-  </si>
-  <si>
-    <t>The page freezes when clicking on the numbers of results</t>
-  </si>
-  <si>
     <t>1 minute</t>
   </si>
   <si>
-    <t>Item sorting</t>
-  </si>
-  <si>
-    <t>Sorting shows accurate information</t>
-  </si>
-  <si>
     <t>2 minutes</t>
   </si>
   <si>
     <t>Moderate severity</t>
-  </si>
-  <si>
-    <t>Click on every sorting option</t>
-  </si>
-  <si>
-    <t>Sorting options show accurate information</t>
-  </si>
-  <si>
-    <t>Best rating and Oldest options return the same data.</t>
   </si>
   <si>
     <t>Account login and registry page test</t>
@@ -289,6 +234,115 @@
   </si>
   <si>
     <t>Egyezik az elvárt eredménnyl.</t>
+  </si>
+  <si>
+    <t>Sikeres regisztráció</t>
+  </si>
+  <si>
+    <t>funkcionális teszt</t>
+  </si>
+  <si>
+    <t>Az alkalmazás fut és elérhető: http://127.0.0.1:8000
+A partner login oldal elérhető: http://127.0.0.1:8000/partner/login
+A „Regisztráljon partnerként” link működik és elérhető a login oldalon
+A tesztben használt e-mail cím még nincs regisztrálva az adatbázisban: zalansimicz@gmail.com</t>
+  </si>
+  <si>
+    <t>Annak ellenőrzése, hogy partnerként történő regisztráció során az űrlap helyes kitöltése után a rendszer sikeresen létrehozza a partner fiókot az e-mail cím megerősítése után, és a felhasználó továbbléphet a dashboardra.</t>
+  </si>
+  <si>
+    <t>2perc</t>
+  </si>
+  <si>
+    <t>Nyisd meg a Partner bejelentkezési oldalt:
+http://127.0.0.1:8000/partner/login
+Kattints a „Regisztráljon partnerként” linkre.
+Töltsd ki a regisztrációs űrlapot az alábbi adatokkal:
+Cég neve: Demo Kft.
+Adószám: 12345678-1-26
+Székhely / cím: 1234 Demo, Demo utca 1.
+Kapcsolattartó neve: Kiss Pista
+Email cím: simiczzalan2005@gmail.com
+Jelszó: 12345678
+Jelszó megerősítése: 12345678
+Kattints a „Regisztráció” gombra.
+Erősítse meg az e-mail címét</t>
+  </si>
+  <si>
+    <t>A regisztráció sikeres.
+A rendszer:
+létrehozza az új partner fiókot az adatbázisban a felhasznalok táblában, illetve a cégek táblában is a hozzá tartozó céget,
+és átirányítja a felhasználót a partner bejelentkezéshez vagy a partner felületre.
+A felhasználó nem kap validációs hibát az űrlapon.</t>
+  </si>
+  <si>
+    <t>Sikeres login</t>
+  </si>
+  <si>
+    <t>Az alkalmazás fut: http://127.0.0.1:8000
+A partner login oldal elérhető:
+http://127.0.0.1:8000/partner/login
+A megadott felhasználó már regisztrálva van az adatbázisban:
+Email: zalansimicz@gmail.com
+Jelszó: 12345678</t>
+  </si>
+  <si>
+    <t>Annak ellenőrzése, hogy a partner felhasználó helyes email és jelszó megadása esetén sikeresen be tud jelentkezni a rendszerbe.</t>
+  </si>
+  <si>
+    <t>1-2perc</t>
+  </si>
+  <si>
+    <t>Nyisd meg a partner login oldalt:
+http://127.0.0.1:8000/partner/login
+Írd be az Email cím mezőbe:
+zalansimicz@gmail.com
+Írd be a Jelszó mezőbe:
+12345678
+Kattints a „Bejelentkezés” gombra.</t>
+  </si>
+  <si>
+    <t>A rendszer elfogadja a bejelentkezési adatokat.
+A felhasználó sikeresen bejelentkezik.
+A rendszer:
+átirányítja a partner dashboard oldalra
+vagy
+Nem jelenik meg hibaüzenet.</t>
+  </si>
+  <si>
+    <t>Sikertelen login</t>
+  </si>
+  <si>
+    <t>validációs teszt</t>
+  </si>
+  <si>
+    <t>Az alkalmazás fut:
+http://127.0.0.1:8000
+A partner login oldal elérhető:
+http://127.0.0.1:8000/partner/login
+A megadott email cím nem létezik a rendszerben, vagy a jelszó hibás</t>
+  </si>
+  <si>
+    <t>Annak ellenőrzése, hogy hibás email cím vagy jelszó megadása esetén:
+a rendszer nem engedi be a felhasználót,
+megfelelő hibaüzenetet jelenít meg,
+a felhasználó a login oldalon marad.</t>
+  </si>
+  <si>
+    <t>Nyisd meg a partner login oldalt:
+http://127.0.0.1:8000/partner/login
+Írd be az Email mezőbe:
+zalansimiczhibas@gmail.com
+Írd be a Jelszó mezőbe:
+1234567
+Kattints a „Bejelentkezés” gombra.</t>
+  </si>
+  <si>
+    <t>A rendszer nem engedi be a felhasználót.
+A login oldalon marad.
+Megjelenik a hibaüzenet:
+„Hibás email cím vagy jelszó”
+Nem történik átirányítás dashboard oldalra.</t>
   </si>
 </sst>
 </file>
@@ -714,8 +768,126 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBA1C781-0C80-4018-8B3B-141250E60562}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.44140625" customWidth="1"/>
+    <col min="2" max="2" width="32.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="203.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="409.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="156.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B1E2F04-C7C7-4BF7-B8B7-53E9F10A00B2}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.33203125" customWidth="1"/>
@@ -731,91 +903,99 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>23</v>
+      <c r="B2" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="92.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="B9" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="34.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>21</v>
+      <c r="B13" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -824,9 +1004,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{222FCA68-CA5A-4081-8552-02095C57CF96}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.33203125" customWidth="1"/>
@@ -842,91 +1022,99 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>22</v>
+      <c r="B2" s="5" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="172.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="63" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="B9" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="156.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="55.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>30</v>
+      <c r="B13" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -934,9 +1122,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3E88C2B-25E3-4285-BF71-6699AB88C669}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -952,91 +1140,99 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="B2" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="156.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="187.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
+      <c r="B9" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="203.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="172.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>38</v>
+      <c r="B13" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1044,7 +1240,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F64FF86E-B3F6-4566-82D1-1C892F185422}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1066,7 +1262,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1074,7 +1270,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1082,7 +1278,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1090,7 +1286,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1098,7 +1294,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1106,7 +1302,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1114,7 +1310,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
@@ -1122,7 +1318,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1130,7 +1326,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1138,7 +1334,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1146,7 +1342,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1154,7 +1350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAA05CFE-9640-4452-8F2B-C16CB83E558A}">
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1176,15 +1372,15 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1192,7 +1388,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1200,7 +1396,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1208,7 +1404,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1216,7 +1412,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1224,7 +1420,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1232,7 +1428,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="94.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1240,7 +1436,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1248,7 +1444,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1256,7 +1452,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1264,7 +1460,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1272,7 +1468,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFB4F6D4-0FF5-4FE1-BD76-CEE9AFE98FEA}">
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1294,15 +1490,15 @@
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1310,7 +1506,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1318,7 +1514,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1326,7 +1522,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1334,7 +1530,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1342,7 +1538,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1350,7 +1546,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="78.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
@@ -1358,7 +1554,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1366,7 +1562,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1374,7 +1570,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1382,7 +1578,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1390,7 +1586,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E94E95F-0233-4D83-B8DD-4AF115CB9958}">
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1412,15 +1608,15 @@
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1428,7 +1624,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="63" thickBot="1" x14ac:dyDescent="0.35">
@@ -1436,7 +1632,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1444,7 +1640,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1452,7 +1648,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1460,7 +1656,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1468,7 +1664,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1476,7 +1672,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1484,7 +1680,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1492,7 +1688,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1500,7 +1696,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1508,7 +1704,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C72E33CD-FB51-4702-A92A-A2C18035FC04}">
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1530,15 +1726,15 @@
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1546,7 +1742,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="63" thickBot="1" x14ac:dyDescent="0.35">
@@ -1554,7 +1750,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1562,7 +1758,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1570,7 +1766,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
@@ -1578,7 +1774,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -1586,7 +1782,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1594,7 +1790,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1602,7 +1798,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="63" thickBot="1" x14ac:dyDescent="0.35">
@@ -1610,7 +1806,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1618,125 +1814,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBA1C781-0C80-4018-8B3B-141250E60562}">
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="27.44140625" customWidth="1"/>
-    <col min="2" max="2" width="32.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="203.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="109.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="409.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="156.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>